<commit_message>
Refresh 2026 season stats from latest GameChanger CSV
Updated through end of season: record 19-8 (was 13-6), team .303
AVG / .834 OPS / 1.47 ERA / 211 K in 176 IP. Top hitters: H. Payne
& H. Smith .375, Hudson Smith .366, Cuda .348, Coray .338. Top
pitchers: Cuda 5-0 / 0.55 ERA / 49 K in 38.1 IP, Bockhorn 5-0 /
1.27 ERA / 49 K in 38.2 IP, Pedersen 5-1 / 1.30 ERA, Bergford 0.00
ERA / 25 K in 12.2 IP. SB: Z. Smith 9, H. Payne 8, Coray 6.

xlsx regenerated via scripts/build_2026_xlsx.py.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Historical/2026/2026_Season_Stats.xlsx
+++ b/Historical/2026/2026_Season_Stats.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y26"/>
+  <dimension ref="A1:Y28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -578,63 +578,63 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="C4" t="n">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>5</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>.217</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>.217</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>.400</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>.617</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
         <v>3</v>
       </c>
-      <c r="F4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G4" t="n">
-        <v>3</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>3</v>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>.214</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>.214</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>.389</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>.603</t>
-        </is>
-      </c>
-      <c r="P4" t="n">
-        <v>2</v>
-      </c>
       <c r="Q4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S4" t="n">
         <v>0</v>
@@ -646,17 +646,17 @@
         <v>3</v>
       </c>
       <c r="V4" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="W4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>.778</t>
+          <t>.857</t>
         </is>
       </c>
     </row>
@@ -667,60 +667,60 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="C5" t="n">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="D5" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E5" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="F5" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="G5" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K5" t="n">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>.242</t>
+          <t>.288</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>.424</t>
+          <t>.492</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>.381</t>
+          <t>.411</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>.805</t>
+          <t>.902</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="Q5" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -735,17 +735,17 @@
         <v>2</v>
       </c>
       <c r="V5" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="W5" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="X5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>.913</t>
+          <t>.927</t>
         </is>
       </c>
     </row>
@@ -756,114 +756,114 @@
         </is>
       </c>
       <c r="B6" t="n">
+        <v>25</v>
+      </c>
+      <c r="C6" t="n">
+        <v>65</v>
+      </c>
+      <c r="D6" t="n">
         <v>17</v>
       </c>
-      <c r="C6" t="n">
-        <v>45</v>
-      </c>
-      <c r="D6" t="n">
-        <v>9</v>
-      </c>
       <c r="E6" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="F6" t="n">
+        <v>18</v>
+      </c>
+      <c r="G6" t="n">
+        <v>20</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>24</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>.338</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>.369</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>.476</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>.845</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>11</v>
+      </c>
+      <c r="R6" t="n">
+        <v>7</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" t="n">
+        <v>1</v>
+      </c>
+      <c r="U6" t="n">
+        <v>6</v>
+      </c>
+      <c r="V6" t="n">
+        <v>29</v>
+      </c>
+      <c r="W6" t="n">
         <v>12</v>
       </c>
-      <c r="G6" t="n">
-        <v>14</v>
-      </c>
-      <c r="H6" t="n">
-        <v>2</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>18</v>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>.356</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>.400</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>.474</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>.874</t>
-        </is>
-      </c>
-      <c r="P6" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>8</v>
-      </c>
-      <c r="R6" t="n">
-        <v>3</v>
-      </c>
-      <c r="S6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T6" t="n">
-        <v>1</v>
-      </c>
-      <c r="U6" t="n">
-        <v>4</v>
-      </c>
-      <c r="V6" t="n">
-        <v>26</v>
-      </c>
-      <c r="W6" t="n">
-        <v>5</v>
-      </c>
       <c r="X6" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>.854</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Spencer Harthorn</t>
+          <t>H Olsen</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -872,33 +872,18 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>9</v>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>.280</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>.360</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>.406</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>.766</t>
+          <t>.000</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -907,52 +892,47 @@
         <v>0</v>
       </c>
       <c r="T7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U7" t="n">
         <v>0</v>
       </c>
       <c r="V7" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="W7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X7" t="n">
-        <v>5</v>
-      </c>
-      <c r="Y7" t="inlineStr">
-        <is>
-          <t>.783</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Kyle Anderson</t>
+          <t>Spencer Harthorn</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
@@ -961,33 +941,33 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>.280</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>.360</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>.406</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>.766</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -996,49 +976,49 @@
         <v>0</v>
       </c>
       <c r="T8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U8" t="n">
         <v>0</v>
       </c>
       <c r="V8" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="W8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="X8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>.783</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Mason Sams</t>
+          <t>Kyle Anderson</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="C9" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
@@ -1050,176 +1030,176 @@
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>.000</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>.000</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>.351</t>
+          <t>.000</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>.685</t>
+          <t>.000</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R9" t="n">
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="T9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V9" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="W9" t="n">
         <v>1</v>
       </c>
       <c r="X9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>.500</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Hudson Smith</t>
+          <t>Mason Sams</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C10" t="n">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="D10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E10" t="n">
+        <v>12</v>
+      </c>
+      <c r="F10" t="n">
+        <v>14</v>
+      </c>
+      <c r="G10" t="n">
+        <v>12</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>12</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>.300</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>.300</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>.318</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>.618</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
         <v>10</v>
       </c>
-      <c r="F10" t="n">
-        <v>8</v>
-      </c>
-      <c r="G10" t="n">
-        <v>8</v>
-      </c>
-      <c r="H10" t="n">
-        <v>1</v>
-      </c>
-      <c r="I10" t="n">
-        <v>1</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="n">
+      <c r="Q10" t="n">
+        <v>2</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" t="n">
+        <v>3</v>
+      </c>
+      <c r="T10" t="n">
+        <v>2</v>
+      </c>
+      <c r="U10" t="n">
+        <v>2</v>
+      </c>
+      <c r="V10" t="n">
         <v>13</v>
       </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>.435</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>.565</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>.556</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>1.121</t>
-        </is>
-      </c>
-      <c r="P10" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>10</v>
-      </c>
-      <c r="R10" t="n">
-        <v>0</v>
-      </c>
-      <c r="S10" t="n">
-        <v>0</v>
-      </c>
-      <c r="T10" t="n">
-        <v>3</v>
-      </c>
-      <c r="U10" t="n">
-        <v>3</v>
-      </c>
-      <c r="V10" t="n">
-        <v>4</v>
-      </c>
       <c r="W10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>.800</t>
+          <t>1.000</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Zach Smith</t>
+          <t>Daniel Vorbete</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="C11" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
@@ -1228,262 +1208,247 @@
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>11</v>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>.188</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>.229</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>.409</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>.638</t>
+          <t>.000</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T11" t="n">
         <v>0</v>
       </c>
       <c r="U11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V11" t="n">
-        <v>113</v>
+        <v>0</v>
       </c>
       <c r="W11" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="X11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>.984</t>
+          <t>.000</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Jack Price</t>
+          <t>Hudson Smith</t>
         </is>
       </c>
       <c r="B12" t="n">
+        <v>19</v>
+      </c>
+      <c r="C12" t="n">
+        <v>41</v>
+      </c>
+      <c r="D12" t="n">
         <v>14</v>
       </c>
-      <c r="C12" t="n">
-        <v>25</v>
-      </c>
-      <c r="D12" t="n">
+      <c r="E12" t="n">
+        <v>15</v>
+      </c>
+      <c r="F12" t="n">
+        <v>12</v>
+      </c>
+      <c r="G12" t="n">
+        <v>12</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" t="n">
+        <v>2</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>20</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>.366</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>.488</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>.538</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>1.026</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>19</v>
+      </c>
+      <c r="R12" t="n">
+        <v>1</v>
+      </c>
+      <c r="S12" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" t="n">
         <v>4</v>
       </c>
-      <c r="E12" t="n">
+      <c r="U12" t="n">
+        <v>4</v>
+      </c>
+      <c r="V12" t="n">
         <v>10</v>
       </c>
-      <c r="F12" t="n">
-        <v>11</v>
-      </c>
-      <c r="G12" t="n">
-        <v>9</v>
-      </c>
-      <c r="H12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" t="n">
-        <v>11</v>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>.400</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>.440</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>.545</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>.985</t>
-        </is>
-      </c>
-      <c r="P12" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>6</v>
-      </c>
-      <c r="R12" t="n">
-        <v>2</v>
-      </c>
-      <c r="S12" t="n">
-        <v>1</v>
-      </c>
-      <c r="T12" t="n">
-        <v>0</v>
-      </c>
-      <c r="U12" t="n">
-        <v>2</v>
-      </c>
-      <c r="V12" t="n">
-        <v>7</v>
-      </c>
       <c r="W12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>.800</t>
+          <t>.909</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Hunter Payne</t>
+          <t>Zach Smith</t>
         </is>
       </c>
       <c r="B13" t="n">
+        <v>27</v>
+      </c>
+      <c r="C13" t="n">
+        <v>71</v>
+      </c>
+      <c r="D13" t="n">
+        <v>24</v>
+      </c>
+      <c r="E13" t="n">
+        <v>16</v>
+      </c>
+      <c r="F13" t="n">
+        <v>17</v>
+      </c>
+      <c r="G13" t="n">
+        <v>11</v>
+      </c>
+      <c r="H13" t="n">
+        <v>4</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" t="n">
+        <v>23</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>.225</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>.324</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>.421</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>.745</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
         <v>19</v>
       </c>
-      <c r="C13" t="n">
-        <v>59</v>
-      </c>
-      <c r="D13" t="n">
-        <v>19</v>
-      </c>
-      <c r="E13" t="n">
-        <v>20</v>
-      </c>
-      <c r="F13" t="n">
-        <v>13</v>
-      </c>
-      <c r="G13" t="n">
-        <v>19</v>
-      </c>
-      <c r="H13" t="n">
-        <v>1</v>
-      </c>
-      <c r="I13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" t="n">
-        <v>21</v>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>.339</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>.356</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>.487</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>.843</t>
-        </is>
-      </c>
-      <c r="P13" t="n">
-        <v>5</v>
-      </c>
       <c r="Q13" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="R13" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="S13" t="n">
         <v>1</v>
       </c>
       <c r="T13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U13" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="V13" t="n">
-        <v>26</v>
+        <v>172</v>
       </c>
       <c r="W13" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="X13" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>.868</t>
+          <t>.990</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Camden Bentley</t>
+          <t>Jack Price</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>18</v>
       </c>
       <c r="C14" t="n">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="D14" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="E14" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F14" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G14" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="H14" t="n">
         <v>1</v>
@@ -1492,51 +1457,51 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>.341</t>
+          <t>.314</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>.432</t>
+          <t>.343</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>.516</t>
+          <t>.455</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>.947</t>
+          <t>.797</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="Q14" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="R14" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="S14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U14" t="n">
         <v>3</v>
       </c>
       <c r="V14" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="W14" t="n">
         <v>1</v>
@@ -1546,389 +1511,389 @@
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>.895</t>
+          <t>.846</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Greyson Riley</t>
+          <t>Hunter Payne</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="C15" t="n">
+        <v>80</v>
+      </c>
+      <c r="D15" t="n">
+        <v>27</v>
+      </c>
+      <c r="E15" t="n">
+        <v>30</v>
+      </c>
+      <c r="F15" t="n">
+        <v>23</v>
+      </c>
+      <c r="G15" t="n">
+        <v>26</v>
+      </c>
+      <c r="H15" t="n">
+        <v>4</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
         <v>34</v>
       </c>
-      <c r="D15" t="n">
-        <v>21</v>
-      </c>
-      <c r="E15" t="n">
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>.375</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>.425</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>.514</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>.939</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>17</v>
+      </c>
+      <c r="R15" t="n">
+        <v>7</v>
+      </c>
+      <c r="S15" t="n">
+        <v>1</v>
+      </c>
+      <c r="T15" t="n">
+        <v>1</v>
+      </c>
+      <c r="U15" t="n">
         <v>8</v>
       </c>
-      <c r="F15" t="n">
-        <v>2</v>
-      </c>
-      <c r="G15" t="n">
+      <c r="V15" t="n">
+        <v>36</v>
+      </c>
+      <c r="W15" t="n">
+        <v>33</v>
+      </c>
+      <c r="X15" t="n">
         <v>7</v>
       </c>
-      <c r="H15" t="n">
-        <v>1</v>
-      </c>
-      <c r="I15" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" t="n">
-        <v>9</v>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>.235</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>.265</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>.491</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>.755</t>
-        </is>
-      </c>
-      <c r="P15" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>13</v>
-      </c>
-      <c r="R15" t="n">
-        <v>5</v>
-      </c>
-      <c r="S15" t="n">
-        <v>1</v>
-      </c>
-      <c r="T15" t="n">
-        <v>1</v>
-      </c>
-      <c r="U15" t="n">
-        <v>2</v>
-      </c>
-      <c r="V15" t="n">
-        <v>21</v>
-      </c>
-      <c r="W15" t="n">
-        <v>0</v>
-      </c>
-      <c r="X15" t="n">
-        <v>2</v>
-      </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>.913</t>
+          <t>.908</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Logan Pedersen</t>
+          <t>Camden Bentley</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>64</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="G16" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>.281</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>.344</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>.457</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>.800</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="Q16" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="R16" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T16" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="U16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="V16" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="W16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="X16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>.946</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Jaxson Knight</t>
+          <t>Greyson Riley</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="C17" t="n">
+        <v>52</v>
+      </c>
+      <c r="D17" t="n">
+        <v>24</v>
+      </c>
+      <c r="E17" t="n">
+        <v>12</v>
+      </c>
+      <c r="F17" t="n">
+        <v>3</v>
+      </c>
+      <c r="G17" t="n">
+        <v>11</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>13</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>.231</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>.250</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>.446</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>.696</t>
+        </is>
+      </c>
+      <c r="P17" t="n">
         <v>9</v>
       </c>
-      <c r="D17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>.000</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>.000</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>.182</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>.182</t>
-        </is>
-      </c>
-      <c r="P17" t="n">
-        <v>2</v>
-      </c>
       <c r="Q17" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="R17" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V17" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="W17" t="n">
         <v>0</v>
       </c>
       <c r="X17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>.935</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Jake Cuda</t>
+          <t>Logan Pedersen</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="C18" t="n">
-        <v>45</v>
+        <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H18" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>.356</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>.578</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>.434</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>1.012</t>
+          <t>2.000</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S18" t="n">
         <v>0</v>
       </c>
       <c r="T18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V18" t="n">
         <v>4</v>
       </c>
       <c r="W18" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="X18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>.857</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Parker Wilson</t>
+          <t>Jaxson Knight</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D19" t="n">
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
@@ -1940,33 +1905,33 @@
         <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>.250</t>
+          <t>.000</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>.250</t>
+          <t>.000</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>.571</t>
+          <t>.182</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>.821</t>
+          <t>.182</t>
         </is>
       </c>
       <c r="P19" t="n">
         <v>2</v>
       </c>
       <c r="Q19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R19" t="n">
         <v>0</v>
@@ -1981,10 +1946,10 @@
         <v>0</v>
       </c>
       <c r="V19" t="n">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="W19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X19" t="n">
         <v>0</v>
@@ -1998,54 +1963,64 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Nathan Cheek</t>
+          <t>Jake Cuda</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="D20" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K20" t="n">
-        <v>0</v>
+        <v>35</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>.348</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>.530</t>
+        </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>.421</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>.951</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q20" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="R20" t="n">
         <v>1</v>
@@ -2054,16 +2029,16 @@
         <v>0</v>
       </c>
       <c r="T20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V20" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="W20" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="X20" t="n">
         <v>0</v>
@@ -2077,29 +2052,29 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Carter Collins</t>
+          <t>Parker Wilson</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="C21" t="n">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="D21" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E21" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G21" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
@@ -2108,36 +2083,36 @@
         <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>.286</t>
+          <t>.200</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>.357</t>
+          <t>.200</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>.429</t>
+          <t>.500</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>.786</t>
+          <t>.700</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="Q21" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="R21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S21" t="n">
         <v>0</v>
@@ -2146,37 +2121,37 @@
         <v>0</v>
       </c>
       <c r="U21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V21" t="n">
-        <v>42</v>
+        <v>7</v>
       </c>
       <c r="W21" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="X21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>.957</t>
+          <t>1.000</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Quentin Bockhorn</t>
+          <t>Nathan Cheek</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C22" t="n">
         <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
@@ -2199,24 +2174,14 @@
       <c r="K22" t="n">
         <v>0</v>
       </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>.000</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>.000</t>
-        </is>
-      </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="P22" t="n">
@@ -2226,7 +2191,7 @@
         <v>0</v>
       </c>
       <c r="R22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S22" t="n">
         <v>0</v>
@@ -2238,46 +2203,46 @@
         <v>0</v>
       </c>
       <c r="V22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W22" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="X22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>.833</t>
+          <t>1.000</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Max Bergford</t>
+          <t>Carter Collins</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>34</v>
       </c>
       <c r="D23" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H23" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
@@ -2286,36 +2251,36 @@
         <v>0</v>
       </c>
       <c r="K23" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>.324</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>.382</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>.500</t>
+          <t>.452</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>.500</t>
+          <t>.835</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q23" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="R23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S23" t="n">
         <v>0</v>
@@ -2324,193 +2289,376 @@
         <v>0</v>
       </c>
       <c r="U23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V23" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="W23" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="X23" t="n">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>.961</t>
+        </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>Quentin Bockhorn</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>0</v>
+      </c>
+      <c r="R24" t="n">
+        <v>0</v>
+      </c>
+      <c r="S24" t="n">
+        <v>0</v>
+      </c>
+      <c r="T24" t="n">
+        <v>0</v>
+      </c>
+      <c r="U24" t="n">
+        <v>0</v>
+      </c>
+      <c r="V24" t="n">
+        <v>1</v>
+      </c>
+      <c r="W24" t="n">
+        <v>4</v>
+      </c>
+      <c r="X24" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>.833</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Max Bergford</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>2</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>.500</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>.500</t>
+        </is>
+      </c>
+      <c r="P25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>1</v>
+      </c>
+      <c r="R25" t="n">
+        <v>0</v>
+      </c>
+      <c r="S25" t="n">
+        <v>0</v>
+      </c>
+      <c r="T25" t="n">
+        <v>0</v>
+      </c>
+      <c r="U25" t="n">
+        <v>0</v>
+      </c>
+      <c r="V25" t="n">
+        <v>0</v>
+      </c>
+      <c r="W25" t="n">
+        <v>1</v>
+      </c>
+      <c r="X25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>Hawken Smith</t>
         </is>
       </c>
-      <c r="B24" t="n">
-        <v>11</v>
-      </c>
-      <c r="C24" t="n">
-        <v>25</v>
-      </c>
-      <c r="D24" t="n">
-        <v>11</v>
-      </c>
-      <c r="E24" t="n">
+      <c r="B26" t="n">
+        <v>14</v>
+      </c>
+      <c r="C26" t="n">
+        <v>32</v>
+      </c>
+      <c r="D26" t="n">
+        <v>14</v>
+      </c>
+      <c r="E26" t="n">
+        <v>12</v>
+      </c>
+      <c r="F26" t="n">
+        <v>15</v>
+      </c>
+      <c r="G26" t="n">
         <v>9</v>
       </c>
-      <c r="F24" t="n">
-        <v>13</v>
-      </c>
-      <c r="G24" t="n">
-        <v>6</v>
-      </c>
-      <c r="H24" t="n">
-        <v>2</v>
-      </c>
-      <c r="I24" t="n">
-        <v>1</v>
-      </c>
-      <c r="J24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" t="n">
-        <v>13</v>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>.360</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>.520</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>.553</t>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>1.073</t>
-        </is>
-      </c>
-      <c r="P24" t="n">
+      <c r="H26" t="n">
+        <v>2</v>
+      </c>
+      <c r="I26" t="n">
+        <v>1</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" t="n">
+        <v>16</v>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>.375</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>.500</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>.551</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>1.051</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
         <v>3</v>
       </c>
-      <c r="Q24" t="n">
-        <v>6</v>
-      </c>
-      <c r="R24" t="n">
-        <v>6</v>
-      </c>
-      <c r="S24" t="n">
-        <v>0</v>
-      </c>
-      <c r="T24" t="n">
-        <v>1</v>
-      </c>
-      <c r="U24" t="n">
-        <v>2</v>
-      </c>
-      <c r="V24" t="n">
-        <v>36</v>
-      </c>
-      <c r="W24" t="n">
+      <c r="Q26" t="n">
+        <v>7</v>
+      </c>
+      <c r="R26" t="n">
+        <v>8</v>
+      </c>
+      <c r="S26" t="n">
+        <v>0</v>
+      </c>
+      <c r="T26" t="n">
+        <v>2</v>
+      </c>
+      <c r="U26" t="n">
+        <v>3</v>
+      </c>
+      <c r="V26" t="n">
+        <v>49</v>
+      </c>
+      <c r="W26" t="n">
         <v>5</v>
       </c>
-      <c r="X24" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y24" t="inlineStr">
+      <c r="X26" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y26" t="inlineStr">
         <is>
           <t>1.000</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>TEAM</t>
         </is>
       </c>
-      <c r="B26" s="3" t="n">
-        <v>19</v>
-      </c>
-      <c r="C26" s="3" t="n">
-        <v>497</v>
-      </c>
-      <c r="D26" s="3" t="n">
-        <v>156</v>
-      </c>
-      <c r="E26" s="3" t="n">
-        <v>152</v>
-      </c>
-      <c r="F26" s="3" t="n">
-        <v>129</v>
-      </c>
-      <c r="G26" s="3" t="n">
-        <v>123</v>
-      </c>
-      <c r="H26" s="3" t="n">
-        <v>22</v>
-      </c>
-      <c r="I26" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J26" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="K26" s="3" t="n">
-        <v>190</v>
-      </c>
-      <c r="L26" s="3" t="inlineStr">
-        <is>
-          <t>.306</t>
-        </is>
-      </c>
-      <c r="M26" s="3" t="inlineStr">
+      <c r="B28" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>704</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>215</v>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>213</v>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>185</v>
+      </c>
+      <c r="G28" s="3" t="n">
+        <v>172</v>
+      </c>
+      <c r="H28" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="I28" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="J28" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="K28" s="3" t="n">
+        <v>269</v>
+      </c>
+      <c r="L28" s="3" t="inlineStr">
+        <is>
+          <t>.303</t>
+        </is>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
         <is>
           <t>.382</t>
         </is>
       </c>
-      <c r="N26" s="3" t="inlineStr">
-        <is>
-          <t>.460</t>
-        </is>
-      </c>
-      <c r="O26" s="3" t="inlineStr">
-        <is>
-          <t>.842</t>
-        </is>
-      </c>
-      <c r="P26" s="3" t="n">
-        <v>95</v>
-      </c>
-      <c r="Q26" s="3" t="n">
-        <v>120</v>
-      </c>
-      <c r="R26" s="3" t="n">
-        <v>34</v>
-      </c>
-      <c r="S26" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="T26" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="U26" s="3" t="n">
-        <v>38</v>
-      </c>
-      <c r="V26" s="3" t="n">
-        <v>375</v>
-      </c>
-      <c r="W26" s="3" t="n">
-        <v>68</v>
-      </c>
-      <c r="X26" s="3" t="n">
-        <v>29</v>
-      </c>
-      <c r="Y26" s="3" t="inlineStr">
-        <is>
-          <t>.939</t>
+      <c r="N28" s="3" t="inlineStr">
+        <is>
+          <t>.452</t>
+        </is>
+      </c>
+      <c r="O28" s="3" t="inlineStr">
+        <is>
+          <t>.834</t>
+        </is>
+      </c>
+      <c r="P28" s="3" t="n">
+        <v>140</v>
+      </c>
+      <c r="Q28" s="3" t="n">
+        <v>160</v>
+      </c>
+      <c r="R28" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="S28" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="T28" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="U28" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="V28" s="3" t="n">
+        <v>528</v>
+      </c>
+      <c r="W28" s="3" t="n">
+        <v>122</v>
+      </c>
+      <c r="X28" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="Y28" s="3" t="inlineStr">
+        <is>
+          <t>.941</t>
         </is>
       </c>
     </row>
@@ -2625,18 +2773,18 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -2645,7 +2793,7 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -2663,7 +2811,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>.750</t>
+          <t>.720</t>
         </is>
       </c>
     </row>
@@ -2674,51 +2822,51 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D5" t="n">
         <v>1</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>15.0</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>23</v>
+        <v>61</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J5" t="n">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="K5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>1.867</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>.500</t>
+          <t>.933</t>
         </is>
       </c>
     </row>
@@ -2794,41 +2942,41 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H7" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J7" t="n">
         <v>8</v>
       </c>
       <c r="K7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="L7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M7" t="n">
         <v>0</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>.955</t>
+          <t>5.250</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>.818</t>
+          <t>1.250</t>
         </is>
       </c>
     </row>
@@ -2894,51 +3042,51 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>20.2</t>
+          <t>32.1</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>91</v>
+        <v>150</v>
       </c>
       <c r="G9" t="n">
+        <v>34</v>
+      </c>
+      <c r="H9" t="n">
         <v>18</v>
       </c>
-      <c r="H9" t="n">
-        <v>11</v>
-      </c>
       <c r="I9" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J9" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="K9" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="L9" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="M9" t="n">
         <v>0</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>1.016</t>
+          <t>1.299</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>1.065</t>
+          <t>1.361</t>
         </is>
       </c>
     </row>
@@ -2949,51 +3097,51 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>28.0</t>
+          <t>38.1</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>110</v>
+        <v>163</v>
       </c>
       <c r="G10" t="n">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="H10" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J10" t="n">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="K10" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="L10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M10" t="n">
         <v>0</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>.548</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>.857</t>
+          <t>1.070</t>
         </is>
       </c>
     </row>
@@ -3007,18 +3155,18 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="G11" t="n">
         <v>2</v>
@@ -3030,10 +3178,10 @@
         <v>5</v>
       </c>
       <c r="J11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -3043,12 +3191,12 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>11.67</t>
+          <t>8.750</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2.333</t>
+          <t>2.000</t>
         </is>
       </c>
     </row>
@@ -3069,41 +3217,41 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="G12" t="n">
+        <v>7</v>
+      </c>
+      <c r="H12" t="n">
+        <v>8</v>
+      </c>
+      <c r="I12" t="n">
         <v>5</v>
-      </c>
-      <c r="H12" t="n">
-        <v>6</v>
-      </c>
-      <c r="I12" t="n">
-        <v>3</v>
       </c>
       <c r="J12" t="n">
         <v>11</v>
       </c>
       <c r="K12" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M12" t="n">
         <v>0</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2.032</t>
+          <t>3.281</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>.774</t>
+          <t>1.125</t>
         </is>
       </c>
     </row>
@@ -3114,7 +3262,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C13" t="n">
         <v>0</v>
@@ -3124,26 +3272,26 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>30.2</t>
+          <t>38.2</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>124</v>
+        <v>160</v>
       </c>
       <c r="G13" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="H13" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I13" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J13" t="n">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="K13" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="L13" t="n">
         <v>2</v>
@@ -3153,12 +3301,12 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>.913</t>
+          <t>1.267</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>1.043</t>
+          <t>1.138</t>
         </is>
       </c>
     </row>
@@ -3169,7 +3317,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C14" t="n">
         <v>1</v>
@@ -3179,14 +3327,14 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>12.2</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>19</v>
+        <v>50</v>
       </c>
       <c r="G14" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H14" t="n">
         <v>3</v>
@@ -3195,10 +3343,10 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="K14" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -3213,7 +3361,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>1.154</t>
+          <t>.868</t>
         </is>
       </c>
     </row>
@@ -3224,51 +3372,51 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>125.0</t>
+          <t>176.0</t>
         </is>
       </c>
       <c r="F16" s="3" t="n">
-        <v>515</v>
+        <v>755</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>72</v>
+        <v>124</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>40</v>
+        <v>69</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>154</v>
+        <v>211</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>49</v>
+        <v>75</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N16" s="3" t="inlineStr">
         <is>
-          <t>.952</t>
+          <t>1.472</t>
         </is>
       </c>
       <c r="O16" s="3" t="inlineStr">
         <is>
-          <t>.968</t>
+          <t>1.131</t>
         </is>
       </c>
     </row>

</xml_diff>